<commit_message>
Updated Work time report
</commit_message>
<xml_diff>
--- a/docs/Työajan seuranta.xlsx
+++ b/docs/Työajan seuranta.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unioulu-my.sharepoint.com/personal/samikkol22_students_oamk_fi/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EBE10E26-9C5F-4C98-B842-FC6001B42ED7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B1E47DA6-5601-4D8D-AB99-07AA9EE9856D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-35760" yWindow="2400" windowWidth="16455" windowHeight="9450" activeTab="2" xr2:uid="{B7036960-D674-4B76-B564-D076AACD5E6B}"/>
+    <workbookView xWindow="-35760" yWindow="2400" windowWidth="16455" windowHeight="9450" firstSheet="2" activeTab="2" xr2:uid="{B7036960-D674-4B76-B564-D076AACD5E6B}"/>
   </bookViews>
   <sheets>
     <sheet name="Riku Ängeslevä" sheetId="4" r:id="rId1"/>
@@ -1544,7 +1544,7 @@
       </c>
       <c r="F2">
         <f>SUM(C3:C139)</f>
-        <v>50.5</v>
+        <v>51.5</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1753,7 +1753,7 @@
         <v>90</v>
       </c>
       <c r="C21">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2230,6 +2230,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="8e13ffe0-cb3e-4b14-846c-c9074a87516f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002C3CF33C597F1D4C8BCF4EB52F57E21C" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8682ee33dd4252813a781844741f1afd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="8e13ffe0-cb3e-4b14-846c-c9074a87516f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0c02225184b8cf34fdc03dd37dcb02cf" ns3:_="">
     <xsd:import namespace="8e13ffe0-cb3e-4b14-846c-c9074a87516f"/>
@@ -2417,25 +2434,8 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="8e13ffe0-cb3e-4b14-846c-c9074a87516f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{88E65DC3-835B-4102-B9E4-1EFEE48C8D75}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1544648-42C0-41A8-A47C-8273BEEEEBBA}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2443,7 +2443,7 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E1544648-42C0-41A8-A47C-8273BEEEEBBA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{88E65DC3-835B-4102-B9E4-1EFEE48C8D75}"/>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>